<commit_message>
finish stra8 counts finally!
</commit_message>
<xml_diff>
--- a/data/raw/Cell_Counts/Stra8_100nMRA/20250104_100nMRA_Stra8_Counts.xlsx
+++ b/data/raw/Cell_Counts/Stra8_100nMRA/20250104_100nMRA_Stra8_Counts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://umhealth-my.sharepoint.com/personal/kbonefas_med_umich_edu/Documents/Documents/KDM5C_Germ_Mechanism/data/raw/Cell_Counts/Stra8_100nMRA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{AB1CBD6F-272E-4ED6-8835-93A1E18BE2BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D64E9C9-9596-4FD5-8A9E-89AA5C4371DC}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="13_ncr:1_{AB1CBD6F-272E-4ED6-8835-93A1E18BE2BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAD2854C-ACF3-4106-83B6-62A4A5AB644F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D4F34921-D08F-4BAD-B6B0-3F60A59243DD}"/>
+    <workbookView xWindow="4800" yWindow="120" windowWidth="14340" windowHeight="8890" xr2:uid="{D4F34921-D08F-4BAD-B6B0-3F60A59243DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -157,6 +157,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1376,6 +1380,12 @@
       <c r="C53" t="s">
         <v>6</v>
       </c>
+      <c r="D53">
+        <v>77</v>
+      </c>
+      <c r="E53">
+        <v>27</v>
+      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
@@ -1387,6 +1397,12 @@
       <c r="C54" t="s">
         <v>6</v>
       </c>
+      <c r="D54">
+        <v>55</v>
+      </c>
+      <c r="E54">
+        <v>40</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
@@ -1398,6 +1414,12 @@
       <c r="C55" t="s">
         <v>6</v>
       </c>
+      <c r="D55">
+        <v>111</v>
+      </c>
+      <c r="E55">
+        <v>47</v>
+      </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
@@ -1409,6 +1431,12 @@
       <c r="C56" t="s">
         <v>6</v>
       </c>
+      <c r="D56">
+        <v>70</v>
+      </c>
+      <c r="E56">
+        <v>53</v>
+      </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
@@ -1420,6 +1448,12 @@
       <c r="C57" t="s">
         <v>6</v>
       </c>
+      <c r="D57">
+        <v>126</v>
+      </c>
+      <c r="E57">
+        <v>69</v>
+      </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
@@ -1431,6 +1465,12 @@
       <c r="C58" t="s">
         <v>6</v>
       </c>
+      <c r="D58">
+        <v>73</v>
+      </c>
+      <c r="E58">
+        <v>31</v>
+      </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
@@ -1442,6 +1482,12 @@
       <c r="C59" t="s">
         <v>6</v>
       </c>
+      <c r="D59">
+        <v>87</v>
+      </c>
+      <c r="E59">
+        <v>36</v>
+      </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
@@ -1453,6 +1499,12 @@
       <c r="C60" t="s">
         <v>6</v>
       </c>
+      <c r="D60">
+        <v>89</v>
+      </c>
+      <c r="E60">
+        <v>48</v>
+      </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
@@ -1464,6 +1516,12 @@
       <c r="C61" t="s">
         <v>6</v>
       </c>
+      <c r="D61">
+        <v>40</v>
+      </c>
+      <c r="E61">
+        <v>22</v>
+      </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
@@ -1611,6 +1669,12 @@
       <c r="C70" t="s">
         <v>6</v>
       </c>
+      <c r="D70">
+        <v>57</v>
+      </c>
+      <c r="E70">
+        <v>35</v>
+      </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
@@ -1622,6 +1686,12 @@
       <c r="C71" t="s">
         <v>6</v>
       </c>
+      <c r="D71">
+        <v>81</v>
+      </c>
+      <c r="E71">
+        <v>31</v>
+      </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
@@ -1633,6 +1703,12 @@
       <c r="C72" t="s">
         <v>6</v>
       </c>
+      <c r="D72">
+        <v>34</v>
+      </c>
+      <c r="E72">
+        <v>10</v>
+      </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
@@ -1763,6 +1839,12 @@
       <c r="C80" t="s">
         <v>6</v>
       </c>
+      <c r="D80">
+        <v>104</v>
+      </c>
+      <c r="E80">
+        <v>46</v>
+      </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
@@ -1774,6 +1856,12 @@
       <c r="C81" t="s">
         <v>6</v>
       </c>
+      <c r="D81">
+        <v>87</v>
+      </c>
+      <c r="E81">
+        <v>43</v>
+      </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
@@ -1785,6 +1873,12 @@
       <c r="C82" t="s">
         <v>6</v>
       </c>
+      <c r="D82">
+        <v>28</v>
+      </c>
+      <c r="E82">
+        <v>19</v>
+      </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
@@ -2901,6 +2995,12 @@
       <c r="C148" t="s">
         <v>19</v>
       </c>
+      <c r="D148">
+        <v>39</v>
+      </c>
+      <c r="E148">
+        <v>1</v>
+      </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
@@ -2912,6 +3012,12 @@
       <c r="C149" t="s">
         <v>19</v>
       </c>
+      <c r="D149">
+        <v>53</v>
+      </c>
+      <c r="E149">
+        <v>0</v>
+      </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
@@ -2923,6 +3029,12 @@
       <c r="C150" t="s">
         <v>19</v>
       </c>
+      <c r="D150">
+        <v>70</v>
+      </c>
+      <c r="E150">
+        <v>0</v>
+      </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
@@ -2933,6 +3045,12 @@
       </c>
       <c r="C151" t="s">
         <v>19</v>
+      </c>
+      <c r="D151">
+        <v>58</v>
+      </c>
+      <c r="E151">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>